<commit_message>
app-a: layout-inference parser — transposed, unnamed specs, index cols
- transposed labeled templates: if 포인트/스펙/상한/하한 sit in one row,
  transpose and reuse the label parser (F03)
- inferLayoutParse/analyzeGrid: finds the numeric block, leading
  text/1..N/serial columns, spec vectors by rank consistency (roles
  assigned by value: max=USL, min=LSL), nearest text row as point names,
  and races original vs transposed by cohesion score (F04/F06/F09/F11)
- ambiguity (small margin or near-square headerless) keeps the runner-up
  as parsed.alt with needPreview for the upcoming preview dialog (F07)
- positionalTemplateParse hardened: all-numeric header rejected, spec
  order validated (usl>lsl, lsl<=spec<=usl) so headerless matrices fall
  through to inference instead of mis-parsing (F09)
- specless files fail with a clear reason toast (F12)

Node chain tests: 22/22 across F01-F12.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/app-a/docs/fixtures/F07-ambiguous-square.xlsx
+++ b/app-a/docs/fixtures/F07-ambiguous-square.xlsx
@@ -12,648 +12,648 @@
   <sheetData>
     <row r="1">
       <c r="A1">
-        <v>10</v>
+        <v>5</v>
       </c>
       <c r="B1">
         <v>10</v>
       </c>
       <c r="C1">
-        <v>10</v>
+        <v>15</v>
       </c>
       <c r="D1">
-        <v>10</v>
+        <v>6</v>
       </c>
       <c r="E1">
-        <v>10</v>
+        <v>7</v>
       </c>
       <c r="F1">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="G1">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="H1">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="I1">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="J1">
-        <v>10</v>
+        <v>13</v>
       </c>
       <c r="K1">
-        <v>10</v>
+        <v>14</v>
       </c>
       <c r="L1">
-        <v>10</v>
+        <v>10.5</v>
       </c>
     </row>
     <row r="2">
       <c r="A2">
-        <v>10.35</v>
+        <v>5.35</v>
       </c>
       <c r="B2">
         <v>10.35</v>
       </c>
       <c r="C2">
-        <v>10.35</v>
+        <v>15.35</v>
       </c>
       <c r="D2">
-        <v>10.35</v>
+        <v>6.35</v>
       </c>
       <c r="E2">
-        <v>10.35</v>
+        <v>7.35</v>
       </c>
       <c r="F2">
-        <v>10.35</v>
+        <v>8.35</v>
       </c>
       <c r="G2">
-        <v>10.35</v>
+        <v>9.35</v>
       </c>
       <c r="H2">
-        <v>10.35</v>
+        <v>11.35</v>
       </c>
       <c r="I2">
-        <v>10.35</v>
+        <v>12.35</v>
       </c>
       <c r="J2">
-        <v>10.35</v>
+        <v>13.35</v>
       </c>
       <c r="K2">
-        <v>10.35</v>
+        <v>14.35</v>
       </c>
       <c r="L2">
-        <v>10.35</v>
+        <v>10.85</v>
       </c>
     </row>
     <row r="3">
       <c r="A3">
-        <v>9.65</v>
+        <v>4.65</v>
       </c>
       <c r="B3">
         <v>9.65</v>
       </c>
       <c r="C3">
-        <v>9.65</v>
+        <v>14.65</v>
       </c>
       <c r="D3">
-        <v>9.65</v>
+        <v>5.65</v>
       </c>
       <c r="E3">
-        <v>9.65</v>
+        <v>6.65</v>
       </c>
       <c r="F3">
-        <v>9.65</v>
+        <v>7.65</v>
       </c>
       <c r="G3">
-        <v>9.65</v>
+        <v>8.65</v>
       </c>
       <c r="H3">
-        <v>9.65</v>
+        <v>10.65</v>
       </c>
       <c r="I3">
-        <v>9.65</v>
+        <v>11.65</v>
       </c>
       <c r="J3">
-        <v>9.65</v>
+        <v>12.65</v>
       </c>
       <c r="K3">
-        <v>9.65</v>
+        <v>13.65</v>
       </c>
       <c r="L3">
-        <v>9.65</v>
+        <v>10.15</v>
       </c>
     </row>
     <row r="4">
       <c r="A4">
-        <v>10.174</v>
+        <v>5.174</v>
       </c>
       <c r="B4">
         <v>10.076</v>
       </c>
       <c r="C4">
-        <v>10.183</v>
+        <v>15.183</v>
       </c>
       <c r="D4">
-        <v>9.87</v>
+        <v>5.87</v>
       </c>
       <c r="E4">
-        <v>9.864</v>
+        <v>6.864</v>
       </c>
       <c r="F4">
-        <v>9.825</v>
+        <v>7.825</v>
       </c>
       <c r="G4">
-        <v>10.148</v>
+        <v>9.148</v>
       </c>
       <c r="H4">
-        <v>9.829</v>
+        <v>10.829</v>
       </c>
       <c r="I4">
-        <v>9.813</v>
+        <v>11.813</v>
       </c>
       <c r="J4">
-        <v>9.88</v>
+        <v>12.88</v>
       </c>
       <c r="K4">
-        <v>9.943</v>
+        <v>13.943</v>
       </c>
       <c r="L4">
-        <v>9.863</v>
+        <v>10.363</v>
       </c>
     </row>
     <row r="5">
       <c r="A5">
-        <v>10.017</v>
+        <v>5.017</v>
       </c>
       <c r="B5">
         <v>9.893</v>
       </c>
       <c r="C5">
-        <v>10.163</v>
+        <v>15.163</v>
       </c>
       <c r="D5">
-        <v>10.016</v>
+        <v>6.016</v>
       </c>
       <c r="E5">
-        <v>10.152</v>
+        <v>7.152</v>
       </c>
       <c r="F5">
-        <v>10.157</v>
+        <v>8.157</v>
       </c>
       <c r="G5">
-        <v>10.109</v>
+        <v>9.109</v>
       </c>
       <c r="H5">
-        <v>9.809</v>
+        <v>10.809</v>
       </c>
       <c r="I5">
-        <v>9.835</v>
+        <v>11.835</v>
       </c>
       <c r="J5">
-        <v>9.896</v>
+        <v>12.896</v>
       </c>
       <c r="K5">
-        <v>10.18</v>
+        <v>14.18</v>
       </c>
       <c r="L5">
-        <v>9.948</v>
+        <v>10.448</v>
       </c>
     </row>
     <row r="6">
       <c r="A6">
-        <v>10.139</v>
+        <v>5.139</v>
       </c>
       <c r="B6">
         <v>9.913</v>
       </c>
       <c r="C6">
-        <v>10.053</v>
+        <v>15.053</v>
       </c>
       <c r="D6">
-        <v>9.892</v>
+        <v>5.892</v>
       </c>
       <c r="E6">
-        <v>10.19</v>
+        <v>7.19</v>
       </c>
       <c r="F6">
-        <v>10.07</v>
+        <v>8.07</v>
       </c>
       <c r="G6">
-        <v>9.867</v>
+        <v>8.867</v>
       </c>
       <c r="H6">
-        <v>10.046</v>
+        <v>11.046</v>
       </c>
       <c r="I6">
-        <v>10.006</v>
+        <v>12.006</v>
       </c>
       <c r="J6">
-        <v>10.153</v>
+        <v>13.153</v>
       </c>
       <c r="K6">
-        <v>10.131</v>
+        <v>14.131</v>
       </c>
       <c r="L6">
-        <v>9.844</v>
+        <v>10.344</v>
       </c>
     </row>
     <row r="7">
       <c r="A7">
-        <v>10.184</v>
+        <v>5.184</v>
       </c>
       <c r="B7">
         <v>9.926</v>
       </c>
       <c r="C7">
-        <v>10.139</v>
+        <v>15.139</v>
       </c>
       <c r="D7">
-        <v>9.87</v>
+        <v>5.87</v>
       </c>
       <c r="E7">
-        <v>9.994</v>
+        <v>6.994</v>
       </c>
       <c r="F7">
-        <v>9.988</v>
+        <v>7.988</v>
       </c>
       <c r="G7">
-        <v>9.831</v>
+        <v>8.831</v>
       </c>
       <c r="H7">
-        <v>10.174</v>
+        <v>11.174</v>
       </c>
       <c r="I7">
-        <v>10.102</v>
+        <v>12.102</v>
       </c>
       <c r="J7">
-        <v>9.993</v>
+        <v>12.993</v>
       </c>
       <c r="K7">
-        <v>9.816</v>
+        <v>13.816</v>
       </c>
       <c r="L7">
-        <v>9.842</v>
+        <v>10.342</v>
       </c>
     </row>
     <row r="8">
       <c r="A8">
-        <v>10.065</v>
+        <v>5.065</v>
       </c>
       <c r="B8">
         <v>10.143</v>
       </c>
       <c r="C8">
-        <v>9.891</v>
+        <v>14.891</v>
       </c>
       <c r="D8">
-        <v>10.12</v>
+        <v>6.12</v>
       </c>
       <c r="E8">
-        <v>10.06</v>
+        <v>7.06</v>
       </c>
       <c r="F8">
-        <v>9.849</v>
+        <v>7.849</v>
       </c>
       <c r="G8">
-        <v>10.025</v>
+        <v>9.025</v>
       </c>
       <c r="H8">
-        <v>10.123</v>
+        <v>11.123</v>
       </c>
       <c r="I8">
-        <v>10.19</v>
+        <v>12.19</v>
       </c>
       <c r="J8">
-        <v>9.921</v>
+        <v>12.921</v>
       </c>
       <c r="K8">
-        <v>9.885</v>
+        <v>13.885</v>
       </c>
       <c r="L8">
-        <v>9.952</v>
+        <v>10.452</v>
       </c>
     </row>
     <row r="9">
       <c r="A9">
-        <v>9.832</v>
+        <v>4.832</v>
       </c>
       <c r="B9">
         <v>9.82</v>
       </c>
       <c r="C9">
-        <v>10.119</v>
+        <v>15.119</v>
       </c>
       <c r="D9">
-        <v>9.808</v>
+        <v>5.808</v>
       </c>
       <c r="E9">
-        <v>10.164</v>
+        <v>7.164</v>
       </c>
       <c r="F9">
-        <v>9.885</v>
+        <v>7.885</v>
       </c>
       <c r="G9">
-        <v>10.007</v>
+        <v>9.007</v>
       </c>
       <c r="H9">
-        <v>9.921</v>
+        <v>10.921</v>
       </c>
       <c r="I9">
-        <v>9.934</v>
+        <v>11.934</v>
       </c>
       <c r="J9">
-        <v>9.893</v>
+        <v>12.893</v>
       </c>
       <c r="K9">
-        <v>9.829</v>
+        <v>13.829</v>
       </c>
       <c r="L9">
-        <v>10.135</v>
+        <v>10.635</v>
       </c>
     </row>
     <row r="10">
       <c r="A10">
-        <v>10.033</v>
+        <v>5.033</v>
       </c>
       <c r="B10">
         <v>9.888</v>
       </c>
       <c r="C10">
-        <v>9.847</v>
+        <v>14.847</v>
       </c>
       <c r="D10">
-        <v>9.824</v>
+        <v>5.824</v>
       </c>
       <c r="E10">
-        <v>9.899</v>
+        <v>6.899</v>
       </c>
       <c r="F10">
-        <v>10.16</v>
+        <v>8.16</v>
       </c>
       <c r="G10">
-        <v>10.16</v>
+        <v>9.16</v>
       </c>
       <c r="H10">
-        <v>10.108</v>
+        <v>11.108</v>
       </c>
       <c r="I10">
-        <v>9.463</v>
+        <v>11.463</v>
       </c>
       <c r="J10">
-        <v>10.172</v>
+        <v>13.172</v>
       </c>
       <c r="K10">
-        <v>10.108</v>
+        <v>14.108</v>
       </c>
       <c r="L10">
-        <v>10.053</v>
+        <v>10.553</v>
       </c>
     </row>
     <row r="11">
       <c r="A11">
-        <v>9.872</v>
+        <v>4.872</v>
       </c>
       <c r="B11">
         <v>10.447</v>
       </c>
       <c r="C11">
-        <v>10.169</v>
+        <v>15.169</v>
       </c>
       <c r="D11">
-        <v>10.081</v>
+        <v>6.081</v>
       </c>
       <c r="E11">
-        <v>9.877</v>
+        <v>6.877</v>
       </c>
       <c r="F11">
-        <v>10.134</v>
+        <v>8.134</v>
       </c>
       <c r="G11">
-        <v>9.811</v>
+        <v>8.811</v>
       </c>
       <c r="H11">
-        <v>9.996</v>
+        <v>10.996</v>
       </c>
       <c r="I11">
-        <v>10.063</v>
+        <v>12.063</v>
       </c>
       <c r="J11">
-        <v>9.953</v>
+        <v>12.953</v>
       </c>
       <c r="K11">
-        <v>9.497</v>
+        <v>13.497</v>
       </c>
       <c r="L11">
-        <v>9.957</v>
+        <v>10.457</v>
       </c>
     </row>
     <row r="12">
       <c r="A12">
-        <v>9.94</v>
+        <v>4.94</v>
       </c>
       <c r="B12">
         <v>10.093</v>
       </c>
       <c r="C12">
-        <v>9.959</v>
+        <v>14.959</v>
       </c>
       <c r="D12">
-        <v>9.924</v>
+        <v>5.924</v>
       </c>
       <c r="E12">
-        <v>9.843</v>
+        <v>6.843</v>
       </c>
       <c r="F12">
-        <v>10.01</v>
+        <v>8.01</v>
       </c>
       <c r="G12">
-        <v>10.076</v>
+        <v>9.076</v>
       </c>
       <c r="H12">
-        <v>10.067</v>
+        <v>11.067</v>
       </c>
       <c r="I12">
-        <v>10.173</v>
+        <v>12.173</v>
       </c>
       <c r="J12">
-        <v>10.163</v>
+        <v>13.163</v>
       </c>
       <c r="K12">
-        <v>9.937</v>
+        <v>13.937</v>
       </c>
       <c r="L12">
-        <v>9.982</v>
+        <v>10.482</v>
       </c>
     </row>
     <row r="13">
       <c r="A13">
-        <v>9.942</v>
+        <v>4.942</v>
       </c>
       <c r="B13">
         <v>10.155</v>
       </c>
       <c r="C13">
-        <v>9.847</v>
+        <v>14.847</v>
       </c>
       <c r="D13">
-        <v>9.947</v>
+        <v>5.947</v>
       </c>
       <c r="E13">
-        <v>9.96</v>
+        <v>6.96</v>
       </c>
       <c r="F13">
-        <v>9.944</v>
+        <v>7.944</v>
       </c>
       <c r="G13">
-        <v>9.888</v>
+        <v>8.888</v>
       </c>
       <c r="H13">
-        <v>9.929</v>
+        <v>10.929</v>
       </c>
       <c r="I13">
-        <v>9.94</v>
+        <v>11.94</v>
       </c>
       <c r="J13">
-        <v>9.89</v>
+        <v>12.89</v>
       </c>
       <c r="K13">
-        <v>10.041</v>
+        <v>14.041</v>
       </c>
       <c r="L13">
-        <v>9.958</v>
+        <v>10.458</v>
       </c>
     </row>
     <row r="14">
       <c r="A14">
-        <v>10.139</v>
+        <v>5.139</v>
       </c>
       <c r="B14">
         <v>9.844</v>
       </c>
       <c r="C14">
-        <v>10.069</v>
+        <v>15.069</v>
       </c>
       <c r="D14">
-        <v>9.461</v>
+        <v>5.461</v>
       </c>
       <c r="E14">
-        <v>9.998</v>
+        <v>6.998</v>
       </c>
       <c r="F14">
-        <v>10.072</v>
+        <v>8.072</v>
       </c>
       <c r="G14">
-        <v>9.818</v>
+        <v>8.818</v>
       </c>
       <c r="H14">
-        <v>9.855</v>
+        <v>10.855</v>
       </c>
       <c r="I14">
-        <v>9.922</v>
+        <v>11.922</v>
       </c>
       <c r="J14">
-        <v>10.077</v>
+        <v>13.077</v>
       </c>
       <c r="K14">
-        <v>9.928</v>
+        <v>13.928</v>
       </c>
       <c r="L14">
-        <v>10.169</v>
+        <v>10.669</v>
       </c>
     </row>
     <row r="15">
       <c r="A15">
-        <v>10.051</v>
+        <v>5.051</v>
       </c>
       <c r="B15">
         <v>10.048</v>
       </c>
       <c r="C15">
-        <v>10.106</v>
+        <v>15.106</v>
       </c>
       <c r="D15">
-        <v>9.824</v>
+        <v>5.824</v>
       </c>
       <c r="E15">
-        <v>9.967</v>
+        <v>6.967</v>
       </c>
       <c r="F15">
-        <v>10.035</v>
+        <v>8.035</v>
       </c>
       <c r="G15">
-        <v>10.024</v>
+        <v>9.024</v>
       </c>
       <c r="H15">
-        <v>10.156</v>
+        <v>11.156</v>
       </c>
       <c r="I15">
-        <v>9.871</v>
+        <v>11.871</v>
       </c>
       <c r="J15">
-        <v>10.139</v>
+        <v>13.139</v>
       </c>
       <c r="K15">
-        <v>9.91</v>
+        <v>13.91</v>
       </c>
       <c r="L15">
-        <v>10.17</v>
+        <v>10.67</v>
       </c>
     </row>
     <row r="16">
       <c r="A16">
-        <v>9.936</v>
+        <v>4.936</v>
       </c>
       <c r="B16">
         <v>9.816</v>
       </c>
       <c r="C16">
-        <v>10.042</v>
+        <v>15.042</v>
       </c>
       <c r="D16">
-        <v>10.114</v>
+        <v>6.114</v>
       </c>
       <c r="E16">
-        <v>9.917</v>
+        <v>6.917</v>
       </c>
       <c r="F16">
-        <v>9.88</v>
+        <v>7.88</v>
       </c>
       <c r="G16">
-        <v>9.976</v>
+        <v>8.976</v>
       </c>
       <c r="H16">
-        <v>9.92</v>
+        <v>10.92</v>
       </c>
       <c r="I16">
-        <v>10.018</v>
+        <v>12.018</v>
       </c>
       <c r="J16">
-        <v>10.036</v>
+        <v>13.036</v>
       </c>
       <c r="K16">
-        <v>9.835</v>
+        <v>13.835</v>
       </c>
       <c r="L16">
-        <v>10.14</v>
+        <v>10.64</v>
       </c>
     </row>
     <row r="17">
       <c r="A17">
-        <v>9.954</v>
+        <v>4.954</v>
       </c>
       <c r="B17">
         <v>9.944</v>
       </c>
       <c r="C17">
-        <v>9.991</v>
+        <v>14.991</v>
       </c>
       <c r="D17">
-        <v>9.979</v>
+        <v>5.979</v>
       </c>
       <c r="E17">
-        <v>9.831</v>
+        <v>6.831</v>
       </c>
       <c r="F17">
-        <v>10.192</v>
+        <v>8.192</v>
       </c>
       <c r="G17">
-        <v>10.14</v>
+        <v>9.14</v>
       </c>
       <c r="H17">
-        <v>10.084</v>
+        <v>11.084</v>
       </c>
       <c r="I17">
-        <v>10.07</v>
+        <v>12.07</v>
       </c>
       <c r="J17">
-        <v>9.961</v>
+        <v>12.961</v>
       </c>
       <c r="K17">
-        <v>10.04</v>
+        <v>14.04</v>
       </c>
       <c r="L17">
-        <v>9.905</v>
+        <v>10.405</v>
       </c>
     </row>
   </sheetData>

</xml_diff>